<commit_message>
fix(q3): unify air index and quantify multibeam thickness bias
</commit_message>
<xml_diff>
--- a/modules/40_q3/figures/editable/origin_templates/data/19_Si参数可辨识性气泡图.xlsx
+++ b/modules/40_q3/figures/editable/origin_templates/data/19_Si参数可辨识性气泡图.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="1" r:id="R5d1ce14204794e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据" sheetId="1" r:id="Ra7f68480fc0648f1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -286,54 +286,351 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>拟合方案(标签)</x:v>
+        <x:v>参数(X)</x:v>
       </x:c>
       <x:c r="B1" s="6" t="str">
-        <x:v>入射角(度)(X)</x:v>
+        <x:v>入射角(度)(颜色分组)</x:v>
       </x:c>
       <x:c r="C1" s="6" t="str">
-        <x:v>RMSE(百分点)(Y)</x:v>
+        <x:v>log10相对灵敏度(Y)</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Jacobian条件数(气泡大小)</x:v>
+        <x:v>最弱右奇异方向权重(气泡面积)</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
-        <x:v>触边参数个数(颜色分组)</x:v>
+        <x:v>边界命中(描边)</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>列归一化条件数(辅助)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>10度Airy</x:v>
+        <x:v>d</x:v>
       </x:c>
       <x:c r="B2" s="2" t="n">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C2" s="2" t="n">
-        <x:v>1.8738296801541603</x:v>
+        <x:v>-0.14457174436800674</x:v>
       </x:c>
       <x:c r="D2" s="2" t="n">
-        <x:v>3.088523429790508</x:v>
+        <x:v>0.3498080501606551</x:v>
       </x:c>
       <x:c r="E2" s="2" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" t="n">
+        <x:v>3.087893962880604</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>15度Airy</x:v>
+        <x:v>n3</x:v>
       </x:c>
       <x:c r="B3" s="2" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="n">
+        <x:v>-0.5661103749896975</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="n">
+        <x:v>0.18301657037934774</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F3" t="n">
+        <x:v>3.087893962880604</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>log10N</x:v>
+      </x:c>
+      <x:c r="B4" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C4" t="n">
+        <x:v>-1.947999026556184</x:v>
+      </x:c>
+      <x:c r="D4" t="n">
+        <x:v>0.3931818157503537</x:v>
+      </x:c>
+      <x:c r="E4" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F4" t="n">
+        <x:v>3.087893962880604</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>log10Gamma_e</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C5" t="n">
+        <x:v>-5.4386202074066725</x:v>
+      </x:c>
+      <x:c r="D5" t="n">
+        <x:v>0.07399356370964347</x:v>
+      </x:c>
+      <x:c r="E5" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" t="n">
+        <x:v>3.087893962880604</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>d</x:v>
+      </x:c>
+      <x:c r="B6" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="C3" s="2" t="n">
-        <x:v>3.3553823523633466</x:v>
-      </x:c>
-      <x:c r="D3" s="2" t="n">
-        <x:v>9.643590292070767</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="n">
-        <x:v>2</x:v>
-      </x:c>
+      <x:c r="C6" t="n">
+        <x:v>-0.039884404320705516</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>0.00898986136638474</x:v>
+      </x:c>
+      <x:c r="E6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F6" t="n">
+        <x:v>9.954363116846206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>n3</x:v>
+      </x:c>
+      <x:c r="B7" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C7" t="n">
+        <x:v>-0.5701977244532084</x:v>
+      </x:c>
+      <x:c r="D7" t="n">
+        <x:v>0.16999822019997343</x:v>
+      </x:c>
+      <x:c r="E7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" t="n">
+        <x:v>9.954363116846206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>log10N</x:v>
+      </x:c>
+      <x:c r="B8" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C8" t="n">
+        <x:v>-8.534106889259487</x:v>
+      </x:c>
+      <x:c r="D8" t="n">
+        <x:v>0.459536087485736</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F8" t="n">
+        <x:v>9.954363116846206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>log10Gamma_e</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C9" t="n">
+        <x:v>-8.567441917932458</x:v>
+      </x:c>
+      <x:c r="D9" t="n">
+        <x:v>0.3614758309479058</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F9" t="n">
+        <x:v>9.954363116846206</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10"/>
+      <x:c r="B10"/>
+      <x:c r="C10"/>
+      <x:c r="D10"/>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>